<commit_message>
Add first three fashion market research dossiers
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +90,12 @@
       <b val="1"/>
       <color rgb="001F3A5F"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="B Zar"/>
+      <b val="1"/>
+      <color rgb="001B6B45"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="17">
@@ -175,7 +181,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -197,11 +203,44 @@
         <color rgb="00D9E0E7"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D9E0E7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E0E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E0E7"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D9E0E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E0E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E0E7"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -290,6 +329,13 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -827,19 +873,19 @@
           <t>پروندهٔ عمیق در صف ۱</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="G8" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="H8" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G8" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H8" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -849,12 +895,12 @@
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>□</t>
+          <t>~</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>پژوهش عمیق و اعتبارسنجی مطابق صف سند مادر</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است.</t>
         </is>
       </c>
     </row>
@@ -884,19 +930,19 @@
           <t>پروندهٔ عمیق در صف ۲</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="G9" s="14" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>□</t>
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H9" s="31" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="I9" s="14" t="inlineStr">
@@ -906,12 +952,12 @@
       </c>
       <c r="J9" s="14" t="inlineStr">
         <is>
-          <t>□</t>
+          <t>~</t>
         </is>
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>پژوهش عمیق و اعتبارسنجی مطابق صف سند مادر</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است.</t>
         </is>
       </c>
     </row>
@@ -941,19 +987,19 @@
           <t>پروندهٔ عمیق در صف ۳</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="G10" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="H10" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G10" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H10" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="I10" s="11" t="inlineStr">
@@ -963,12 +1009,12 @@
       </c>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>□</t>
+          <t>~</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>پژوهش عمیق و اعتبارسنجی مطابق صف سند مادر</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است.</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3380,7 @@
           <t>reports/fashion_market_research_master_v0.docx</t>
         </is>
       </c>
-      <c r="C14" s="27" t="n"/>
+      <c r="C14" s="32" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
       <c r="A15" s="28" t="inlineStr">
@@ -3347,7 +3393,7 @@
           <t>methodology/استاندارد_تدوین_گزارش_تحقیقات_بازار_فرصت‌های_فشن.md</t>
         </is>
       </c>
-      <c r="C15" s="29" t="n"/>
+      <c r="C15" s="32" t="n"/>
     </row>
     <row r="16" ht="26" customHeight="1">
       <c r="A16" s="26" t="inlineStr">
@@ -3360,7 +3406,7 @@
           <t>research/fashion_research_status.md</t>
         </is>
       </c>
-      <c r="C16" s="27" t="n"/>
+      <c r="C16" s="32" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Add F-04 and F-05 fashion market dossiers
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ صفر | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۰٫۳ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -769,12 +769,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>اولویت پایین: 2</t>
+          <t>اولویت پایین: 1</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>رد/آرشیوی: 30</t>
+          <t>رد/آرشیوی: 31</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr">
@@ -1018,7 +1018,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="42" customHeight="1">
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
           <t>F-04</t>
@@ -1039,24 +1039,24 @@
           <t>Watch / نیازمند اثبات</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
-        <is>
-          <t>پروندهٔ عمیق در صف ۴</t>
-        </is>
-      </c>
-      <c r="F11" s="14" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="G11" s="14" t="inlineStr">
-        <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>□</t>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۳</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G11" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="I11" s="14" t="inlineStr">
@@ -1066,16 +1066,16 @@
       </c>
       <c r="J11" s="14" t="inlineStr">
         <is>
-          <t>□</t>
-        </is>
-      </c>
-      <c r="K11" s="15" t="inlineStr">
-        <is>
-          <t>پژوهش عمیق و اعتبارسنجی مطابق صف سند مادر</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="42" customHeight="1">
+          <t>~</t>
+        </is>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
           <t>F-05</t>
@@ -1091,29 +1091,29 @@
           <t>B2B</t>
         </is>
       </c>
-      <c r="D12" s="17" t="inlineStr">
-        <is>
-          <t>اولویت پایین</t>
+      <c r="D12" s="19" t="inlineStr">
+        <is>
+          <t>رد / آرشیوی (desk)</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ آرشیوی تصمیم</t>
-        </is>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="G12" s="11" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۳؛ آرشیوی</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
@@ -1123,12 +1123,12 @@
       </c>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>□</t>
+          <t>~</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>تکمیل پروندهٔ آرشیوی؛ بازپیشنهاد نشود مگر فرض بنیادی تغییر کند</t>
+          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add F-06 archive and condition research dossier
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۰٫۳ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۰٫۴ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -769,12 +769,12 @@
       </c>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>اولویت پایین: 1</t>
+          <t>اولویت پایین: 0</t>
         </is>
       </c>
       <c r="I4" s="7" t="inlineStr">
         <is>
-          <t>رد/آرشیوی: 31</t>
+          <t>رد/آرشیوی: 32</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr">
@@ -1132,7 +1132,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="42" customHeight="1">
+    <row r="13" ht="50" customHeight="1">
       <c r="A13" s="14" t="inlineStr">
         <is>
           <t>F-06</t>
@@ -1140,7 +1140,7 @@
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>بایگانی، امانت و condition report لباس آرشیوی/موزه‌ای</t>
+          <t>آرشیو، امانت و condition report لباس</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
@@ -1148,29 +1148,29 @@
           <t>B2B</t>
         </is>
       </c>
-      <c r="D13" s="17" t="inlineStr">
-        <is>
-          <t>زیر‌بخش مسیر F-02</t>
+      <c r="D13" s="19" t="inlineStr">
+        <is>
+          <t>رد / آرشیوی (desk)</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>پوشش در پرونده F-02</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="G13" s="14" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>□</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۴؛ sub-segment F-02</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G13" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H13" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="I13" s="14" t="inlineStr">
@@ -1180,12 +1180,12 @@
       </c>
       <c r="J13" s="14" t="inlineStr">
         <is>
-          <t>□</t>
+          <t>~</t>
         </is>
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>تکمیل پروندهٔ آرشیوی؛ بازپیشنهاد نشود مگر فرض بنیادی تغییر کند</t>
+          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add F-07 social fashion game research dossier
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۰٫۴ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۰٫۵ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="42" customHeight="1">
+    <row r="14" ht="48" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
           <t>F-07</t>
@@ -1212,22 +1212,22 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ آرشیوی؛ بازگشایی فقط با درخواست صریح</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="G14" s="11" t="inlineStr">
-        <is>
-          <t>~</t>
-        </is>
-      </c>
-      <c r="H14" s="11" t="inlineStr">
-        <is>
-          <t>□</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۵؛ Pause</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="H14" s="30" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
@@ -1237,12 +1237,12 @@
       </c>
       <c r="J14" s="11" t="inlineStr">
         <is>
-          <t>□</t>
+          <t>~</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>بازگشایی فقط با درخواست صریح کاربر و trigger ثبت‌شده</t>
+          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Standardize F-01 to F-07 market research structure
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۰٫۵ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۰٫۶ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق در صف ۱</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ hierarchy استاندارد بازآرایی شد</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق در صف ۲</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ hierarchy استاندارد بازآرایی شد</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق در صف ۳</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ hierarchy استاندارد بازآرایی شد</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۳</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ Watch</t>
         </is>
       </c>
       <c r="F11" s="30" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است.</t>
+          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۳؛ آرشیوی</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ آرشیوی</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند.</t>
+          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۴؛ sub-segment F-02</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ sub-segment F-02 / آرشیوی</t>
         </is>
       </c>
       <c r="F13" s="30" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند.</t>
+          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۵؛ Pause</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ Pause</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود.</t>
+          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
         </is>
       </c>
     </row>
@@ -3268,12 +3268,12 @@
       </c>
       <c r="B5" s="24" t="inlineStr">
         <is>
-          <t>مرور/شواهد اولیه موجود</t>
+          <t>مرور/شواهد اولیه موجود؛ dossier desk-research با ساختار استاندارد بازآرایی شده است</t>
         </is>
       </c>
       <c r="C5" s="24" t="inlineStr">
         <is>
-          <t>به معنی پروندهٔ کامل یا توصیهٔ سرمایه‌گذاری نیست.</t>
+          <t>به معنی پژوهش اولیه، پروندهٔ primary-validated یا توصیهٔ سرمایه‌گذاری نیست.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deepen desk research for F-01 and F-02
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۰٫۶ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۰٫۸ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ hierarchy استاندارد بازآرایی شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۸؛ desk-research واقعی F-01 تکمیل شد</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-01: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است.</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ hierarchy استاندارد بازآرایی شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۸؛ desk-research واقعی F-02 تکمیل شد</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-02: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Deepen desk research for F-03 to F-07
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۰٫۸ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۰٫۹ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ hierarchy استاندارد بازآرایی شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ desk-research واقعی F-03 تکمیل شد</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-03: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ Watch</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ desk-research واقعی F-04 تکمیل شد</t>
         </is>
       </c>
       <c r="F11" s="30" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
+          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-04: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ آرشیوی</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ آرشیوی؛ بازبینی واقعی F-05</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
+          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-05: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ sub-segment F-02 / آرشیوی</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ آرشیوی؛ بازبینی واقعی F-06</t>
         </is>
       </c>
       <c r="F13" s="30" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
+          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-06: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۶؛ Pause</t>
+          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ Pause؛ بازبینی واقعی F-07</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد.</t>
+          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-07: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add verifiable local evidence to fashion dossiers
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۰٫۹ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۱٫۰ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۸؛ desk-research واقعی F-01 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-01 تکمیل شد</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
@@ -927,7 +927,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۸؛ desk-research واقعی F-02 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-02 تکمیل شد</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ desk-research واقعی F-03 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-03 تکمیل شد</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ desk-research واقعی F-04 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-04 تکمیل شد</t>
         </is>
       </c>
       <c r="F11" s="30" t="inlineStr">
@@ -1098,7 +1098,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ آرشیوی؛ بازبینی واقعی F-05</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ آرشیوی؛ بازبینی واقعی F-05</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ آرشیوی؛ بازبینی واقعی F-06</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ آرشیوی؛ بازبینی واقعی F-06</t>
         </is>
       </c>
       <c r="F13" s="30" t="inlineStr">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۰٫۹؛ Pause؛ بازبینی واقعی F-07</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ Pause؛ بازبینی واقعی F-07</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Deepen source-level research for all fashion dossiers
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -747,7 +747,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۱٫۰ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۱٫۱ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-01 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-01 تکمیل شد</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-01: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-01: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F01-S17: مرز رسمی social-commerce/شناسهٔ پوشاک ثبت شد؛ گردش نمونه به marketplace تبدیل نشود.</t>
         </is>
       </c>
     </row>
@@ -927,7 +927,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-02 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-02 تکمیل شد</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-02: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-02: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F02-S12: costume/production-document archive دیده شد؛ production WTP یا continuity pain ثابت نشد.</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-03 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-03 تکمیل شد</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
@@ -1014,7 +1014,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-03: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-03: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F03-S17: substitute محلی برای BOM/QC/factory-control ثبت شد؛ tech-pack/version hand-off تنها wedge قابل آزمون است.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ desk-research واقعی F-04 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-04 تکمیل شد</t>
         </is>
       </c>
       <c r="F11" s="30" t="inlineStr">
@@ -1071,7 +1071,7 @@
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-04: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
+          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-04: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F04-S12: قانون مالکیت صنعتی ۲۰۲۴ به ledger افزوده شد؛ certificate ضمانت حقوقی نیست.</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ آرشیوی؛ بازبینی واقعی F-05</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ آرشیوی؛ بازبینی واقعی F-05</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
@@ -1128,7 +1128,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-05: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
+          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-05: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F05-S10: cohort ۲۰+ شعبه و incumbent محلی دیده شد؛ VM-specific failure/WTP همچنان نامعلوم است.</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ آرشیوی؛ بازبینی واقعی F-06</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ آرشیوی؛ بازبینی واقعی F-06</t>
         </is>
       </c>
       <c r="F13" s="30" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-06: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
+          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-06: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F06-S09: governance رسمی اموال فرهنگی counter-thesis را تقویت کرد؛ TAM/procurement ثابت نشده است.</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۰؛ Pause؛ بازبینی واقعی F-07</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ Pause؛ بازبینی واقعی F-07</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-07: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است.</t>
+          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-07: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F07-S13: پیمایش ملی ۱۴۰۲ context موبایل را تازه کرد؛ genre/retention/payer فشن‌گیم نامعلوم است.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add evidence-first market sizing and primary research protocol
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="دفتر کنترل پرونده‌ها" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="راهنما و وضعیت" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="پیوند دفتر اندازه بازار" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'دفتر کنترل پرونده‌ها'!$A$7:$K$48</definedName>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,8 +98,23 @@
       <color rgb="001B6B45"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="B Zar"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="B Zar"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="B Zar"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -180,8 +196,18 @@
         <fgColor rgb="00E8EAED"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -236,11 +262,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7C9D6"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7C9D6"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7C9D6"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7C9D6"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -336,6 +376,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -747,7 +796,7 @@
     <row r="2" ht="25" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>نسخهٔ ۱٫۱ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
+          <t>نسخهٔ ۱٫۲ | شامل همهٔ مسیرهای فعال، Watch، Pause، ردشده و خارج از دامنه در حوزهٔ مد، پوشاک و فشن</t>
         </is>
       </c>
     </row>
@@ -870,7 +919,7 @@
       </c>
       <c r="E8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-01 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۲؛ desk-research واقعی F-01 تکمیل شد</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
@@ -900,7 +949,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-01: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F01-S17: مرز رسمی social-commerce/شناسهٔ پوشاک ثبت شد؛ گردش نمونه به marketplace تبدیل نشود.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-01: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F01-S17: مرز رسمی social-commerce/شناسهٔ پوشاک ثبت شد؛ گردش نمونه به marketplace تبدیل نشود. | نسخهٔ ۱٫۲: دفتر TAM/SAM/SOM افزوده شد؛ بدون denominator واجد و قیمت محلی، مبلغ «محاسبه‌نشده» است.</t>
         </is>
       </c>
     </row>
@@ -927,7 +976,7 @@
       </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-02 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۲؛ desk-research واقعی F-02 تکمیل شد</t>
         </is>
       </c>
       <c r="F9" s="31" t="inlineStr">
@@ -957,7 +1006,7 @@
       </c>
       <c r="K9" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-02: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F02-S12: costume/production-document archive دیده شد؛ production WTP یا continuity pain ثابت نشد.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-02: بازبینی واقعی منابع رسمی جهانی/ایران، محدودیت evidence و گیت پژوهش اولیه در نسخهٔ ۰٫۸ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F02-S12: costume/production-document archive دیده شد؛ production WTP یا continuity pain ثابت نشد. | نسخهٔ ۱٫۲: دفتر TAM/SAM/SOM افزوده شد؛ بدون denominator واجد و قیمت محلی، مبلغ «محاسبه‌نشده» است.</t>
         </is>
       </c>
     </row>
@@ -984,7 +1033,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-03 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۲؛ desk-research واقعی F-03 تکمیل شد</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
@@ -1014,7 +1063,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-03: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F03-S17: substitute محلی برای BOM/QC/factory-control ثبت شد؛ tech-pack/version hand-off تنها wedge قابل آزمون است.</t>
+          <t>پروندهٔ desk-research، منابع و گیت اعتبارسنجی به سند مادر افزوده شد؛ پژوهش اولیه/paid pilot باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-03: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F03-S17: substitute محلی برای BOM/QC/factory-control ثبت شد؛ tech-pack/version hand-off تنها wedge قابل آزمون است. | نسخهٔ ۱٫۲: دفتر TAM/SAM/SOM افزوده شد؛ بدون denominator واجد و قیمت محلی، مبلغ «محاسبه‌نشده» است.</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1090,7 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ desk-research واقعی F-04 تکمیل شد</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۲؛ desk-research واقعی F-04 تکمیل شد</t>
         </is>
       </c>
       <c r="F11" s="30" t="inlineStr">
@@ -1071,7 +1120,7 @@
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-04: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F04-S12: قانون مالکیت صنعتی ۲۰۲۴ به ledger افزوده شد؛ certificate ضمانت حقوقی نیست.</t>
+          <t>پروندهٔ desk-research، ledger و hard-kill ثبت شد؛ WTP، agreement کارشناس، legal review و micro-pilot پرداختی باقی است. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-04: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F04-S12: قانون مالکیت صنعتی ۲۰۲۴ به ledger افزوده شد؛ certificate ضمانت حقوقی نیست. | نسخهٔ ۱٫۲: دفتر TAM/SAM/SOM افزوده شد؛ بدون denominator واجد و قیمت محلی، مبلغ «محاسبه‌نشده» است.</t>
         </is>
       </c>
     </row>
@@ -1098,7 +1147,7 @@
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ آرشیوی؛ بازبینی واقعی F-05</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۲؛ آرشیوی؛ بازبینی واقعی F-05</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
@@ -1128,7 +1177,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-05: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F05-S10: cohort ۲۰+ شعبه و incumbent محلی دیده شد؛ VM-specific failure/WTP همچنان نامعلوم است.</t>
+          <t>دossier desk-research تکمیل شد؛ substituteهای مستقیم ایران مانع تمایز platform-level‌اند. بازپیشنهاد نشود مگر trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-05: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F05-S10: cohort ۲۰+ شعبه و incumbent محلی دیده شد؛ VM-specific failure/WTP همچنان نامعلوم است. | نسخهٔ ۱٫۲: دفتر TAM/SAM/SOM افزوده شد؛ بدون denominator واجد و قیمت محلی، مبلغ «محاسبه‌نشده» است.</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1204,7 @@
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ آرشیوی؛ بازبینی واقعی F-06</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۲؛ آرشیوی؛ بازبینی واقعی F-06</t>
         </is>
       </c>
       <c r="F13" s="30" t="inlineStr">
@@ -1185,7 +1234,7 @@
       </c>
       <c r="K13" s="15" t="inlineStr">
         <is>
-          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-06: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F06-S09: governance رسمی اموال فرهنگی counter-thesis را تقویت کرد؛ TAM/procurement ثابت نشده است.</t>
+          <t>دossier desk-research کامل شد؛ CMSهای موزه‌ای/سامانه‌های ایران و overlap با F-02، مسیر را رد/آرشیوی می‌کند. بازگشایی فقط با trigger مستند. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-06: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F06-S09: governance رسمی اموال فرهنگی counter-thesis را تقویت کرد؛ TAM/procurement ثابت نشده است. | نسخهٔ ۱٫۲: دفتر TAM/SAM/SOM افزوده شد؛ بدون denominator واجد و قیمت محلی، مبلغ «محاسبه‌نشده» است.</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1261,7 @@
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ عمیق نسخهٔ ۱٫۱؛ Pause؛ بازبینی واقعی F-07</t>
+          <t>پروندهٔ عمیق نسخهٔ ۱٫۲؛ Pause؛ بازبینی واقعی F-07</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
@@ -1242,7 +1291,7 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-07: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F07-S13: پیمایش ملی ۱۴۰۲ context موبایل را تازه کرد؛ genre/retention/payer فشن‌گیم نامعلوم است.</t>
+          <t>dossier desk-research کامل شد؛ Pause به درخواست کاربر پابرجاست. هیچ build/pilot بدون reversal صریح انجام نمی‌شود. | عنوان‌ها و hierarchy استاندارد گزارش تحقیقات بازار در نسخهٔ ۰٫۶ بازآرایی شد؛ سطح شواهد و وضعیت تصمیم تغییری نکرد. | F-07: بازبینی واقعی sourceهای رسمی/محلی، limitation و گیت تصمیم در نسخهٔ ۰٫۹ افزوده شد؛ primary research انجام نشده است. | نسخهٔ ۱٫۱: F07-S13: پیمایش ملی ۱۴۰۲ context موبایل را تازه کرد؛ genre/retention/payer فشن‌گیم نامعلوم است. | نسخهٔ ۱٫۲: دفتر TAM/SAM/SOM افزوده شد؛ بدون denominator واجد و قیمت محلی، مبلغ «محاسبه‌نشده» است.</t>
         </is>
       </c>
     </row>
@@ -3418,4 +3467,104 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>وضعیت sizing / نسخهٔ ۱٫۲</t>
+        </is>
+      </c>
+      <c r="B1" s="33" t="inlineStr"/>
+      <c r="C1" s="33" t="inlineStr"/>
+      <c r="D1" s="33" t="inlineStr"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>فایل مکمل</t>
+        </is>
+      </c>
+      <c r="B2" s="34" t="inlineStr">
+        <is>
+          <t>reports/portfolio_TAM_SAM_SOM_evidence_register_1405.xlsx</t>
+        </is>
+      </c>
+      <c r="C2" s="34" t="inlineStr"/>
+      <c r="D2" s="34" t="inlineStr"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>قاعده</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>بدون denominator واجد + قیمت/ARPA محلی، TAM/SAM/SOM پولی محاسبه نمی‌شود.</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr"/>
+      <c r="D3" s="35" t="inlineStr"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>F-01 تا F-06</t>
+        </is>
+      </c>
+      <c r="B4" s="34" t="inlineStr">
+        <is>
+          <t>همهٔ خروجی‌های پولی Uncomputed؛ anchor خارجی فقط برای scope/pricing category است.</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="inlineStr"/>
+      <c r="D4" s="34" t="inlineStr"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>F-07</t>
+        </is>
+      </c>
+      <c r="B5" s="35" t="inlineStr">
+        <is>
+          <t>~31.1M gamer context و 520B تومان Myket proxy؛ هیچ‌کدام TAM/forecast فشن‌گیم نیست.</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr"/>
+      <c r="D5" s="35" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="34" t="inlineStr">
+        <is>
+          <t>primary research</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>instrument آماده شده؛ هیچ اجرا/نمونه/نتیجه‌ای ادعا نشده است.</t>
+        </is>
+      </c>
+      <c r="C6" s="34" t="inlineStr"/>
+      <c r="D6" s="34" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Start 41-report fashion market research master
</commit_message>
<xml_diff>
--- a/reports/fashion_research_portfolio_register_1405.xlsx
+++ b/reports/fashion_research_portfolio_register_1405.xlsx
@@ -1318,7 +1318,7 @@
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>پروندهٔ آرشیوی؛ بازگشایی فقط با درخواست صریح</t>
+          <t>پروندهٔ مستقل اولیه نسخهٔ ۰٫۱؛ پژوهش پایهٔ واقعی در گزارش ۴۱ فرصت شروع شد</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
@@ -1348,7 +1348,7 @@
       </c>
       <c r="K15" s="15" t="inlineStr">
         <is>
-          <t>بازگشایی فقط با درخواست صریح کاربر و trigger ثبت‌شده</t>
+          <t>بازگشایی فقط با درخواست صریح کاربر و trigger ثبت‌شده | نسخهٔ کاری ۰٫۱: پروندهٔ مستقل، منبع خارجی/ایران و مدل اولیهٔ بازار ساخته شد؛ پژوهش اولیه اجرا نشده است.</t>
         </is>
       </c>
     </row>
@@ -1375,7 +1375,7 @@
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>پروندهٔ آرشیوی؛ بازگشایی فقط با درخواست صریح</t>
+          <t>پروندهٔ مستقل اولیه نسخهٔ ۰٫۱؛ پژوهش پایهٔ واقعی در گزارش ۴۱ فرصت شروع شد</t>
         </is>
       </c>
       <c r="F16" s="11" t="inlineStr">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>بازگشایی فقط با درخواست صریح کاربر و trigger ثبت‌شده</t>
+          <t>بازگشایی فقط با درخواست صریح کاربر و trigger ثبت‌شده | نسخهٔ کاری ۰٫۱: پروندهٔ مستقل، منبع خارجی/ایران و مدل اولیهٔ بازار ساخته شد؛ پژوهش اولیه اجرا نشده است.</t>
         </is>
       </c>
     </row>

</xml_diff>